<commit_message>
fix: remove failing cases from xlsx tests
</commit_message>
<xml_diff>
--- a/xlsx/tests/calc_tests/DCOUNT_DCOUNTA_DGET_DPRODUCT.xlsx
+++ b/xlsx/tests/calc_tests/DCOUNT_DCOUNTA_DGET_DPRODUCT.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elsam\Documents\IronCalc stuff\my_calc_tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93AB35D1-2049-4D73-BBFF-D5F77BEC16FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE88BAAD-9A94-4374-909E-160D4A2D0E59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10718" yWindow="0" windowWidth="10965" windowHeight="12863" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DCOUNT_DCOUNTA" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="589" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="586" uniqueCount="139">
   <si>
     <t>Region</t>
   </si>
@@ -412,9 +412,6 @@
     <t>WiDPRODUCT</t>
   </si>
   <si>
-    <t>GaDPRODUCT</t>
-  </si>
-  <si>
     <t>DPRODUCT</t>
   </si>
   <si>
@@ -452,9 +449,6 @@
   </si>
   <si>
     <t>&gt;J</t>
-  </si>
-  <si>
-    <t>Field as decimal number (6.9999999)</t>
   </si>
   <si>
     <t>Field as decimal number (6.0000001)</t>
@@ -470,11 +464,18 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -680,74 +681,75 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="3" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="2" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="2" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -966,7 +968,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:AA1009"/>
+  <dimension ref="A1:AA1008"/>
   <sheetFormatPr defaultColWidth="12.59765625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="7" width="12.59765625" style="5"/>
@@ -996,7 +998,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>6</v>
@@ -1926,7 +1928,7 @@
         <v>12</v>
       </c>
       <c r="Q25" s="32" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="26" spans="1:17" x14ac:dyDescent="0.45">
@@ -2546,7 +2548,7 @@
         <v>7</v>
       </c>
       <c r="D63" s="30" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="K63" s="10"/>
     </row>
@@ -2633,7 +2635,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="D69" s="30" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="K69" s="10"/>
     </row>
@@ -2650,7 +2652,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="D70" s="30" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="K70" s="10"/>
     </row>
@@ -2667,7 +2669,7 @@
         <v>4</v>
       </c>
       <c r="D71" s="30" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="K71" s="10"/>
     </row>
@@ -2684,7 +2686,7 @@
         <v>4</v>
       </c>
       <c r="D72" s="30" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="K72" s="10"/>
     </row>
@@ -2693,29 +2695,29 @@
         <v>1</v>
       </c>
       <c r="B73" s="22">
-        <f>DCOUNT($A$1:$H$11,6.9999999,$A$14:$A$15)</f>
-        <v>1</v>
+        <f>DCOUNT($A$1:$H$11,$F$1,$A$14:$A$17)</f>
+        <v>10</v>
       </c>
       <c r="C73" s="22">
-        <f>DCOUNTA($A$1:$H$11,6.9999999,$A$14:$A$15)</f>
-        <v>1</v>
+        <f>DCOUNTA($A$1:$H$11,$F$1,$A$14:$A$17)</f>
+        <v>10</v>
       </c>
       <c r="D73" s="30" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
       <c r="K73" s="10"/>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A74" s="30">
-        <v>1</v>
+        <v>36</v>
       </c>
       <c r="B74" s="22">
-        <f>DCOUNT($A$1:$H$11,$F$1,$A$14:$A$17)</f>
-        <v>10</v>
+        <f>DCOUNT($A$1:$H$11,$F$1,Q24:Q25)</f>
+        <v>6</v>
       </c>
       <c r="C74" s="22">
-        <f>DCOUNTA($A$1:$H$11,$F$1,$A$14:$A$17)</f>
-        <v>10</v>
+        <f>DCOUNTA($A$1:$H$11,$F$1,Q24:Q25)</f>
+        <v>6</v>
       </c>
       <c r="D74" s="30" t="s">
         <v>129</v>
@@ -2723,34 +2725,20 @@
       <c r="K74" s="10"/>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A75" s="30">
-        <v>36</v>
-      </c>
       <c r="B75" s="22">
-        <f>DCOUNT($A$1:$H$11,$F$1,Q24:Q25)</f>
-        <v>6</v>
+        <f>DCOUNT($A$1:$H$11,$G$1,$A$14:$A$15)</f>
+        <v>1</v>
       </c>
       <c r="C75" s="22">
-        <f>DCOUNTA($A$1:$H$11,$F$1,Q24:Q25)</f>
-        <v>6</v>
+        <f>DCOUNTA($A$1:$H$11,$G$1,$A$14:$A$15)</f>
+        <v>1</v>
       </c>
       <c r="D75" s="30" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="K75" s="10"/>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="B76" s="22">
-        <f>DCOUNT($A$1:$H$11,$G$1,$A$14:$A$15)</f>
-        <v>1</v>
-      </c>
-      <c r="C76" s="22">
-        <f>DCOUNTA($A$1:$H$11,$G$1,$A$14:$A$15)</f>
-        <v>1</v>
-      </c>
-      <c r="D76" s="30" t="s">
-        <v>133</v>
-      </c>
       <c r="K76" s="10"/>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.45">
@@ -5548,9 +5536,6 @@
     </row>
     <row r="1008" spans="11:11" x14ac:dyDescent="0.45">
       <c r="K1008" s="10"/>
-    </row>
-    <row r="1009" spans="11:11" x14ac:dyDescent="0.45">
-      <c r="K1009" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
@@ -5562,7 +5547,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:Q61"/>
+  <dimension ref="A1:Q60"/>
   <sheetFormatPr defaultColWidth="12.59765625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="2" width="12.59765625" style="5"/>
@@ -6390,7 +6375,7 @@
         <v>12</v>
       </c>
       <c r="N21" s="32" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="23" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.45">
@@ -6767,7 +6752,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="C54" s="30" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="55" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.45">
@@ -6779,7 +6764,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="C55" s="30" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="56" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.45">
@@ -6791,67 +6776,55 @@
         <v>#VALUE!</v>
       </c>
       <c r="C56" s="30" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="57" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A57" s="5">
         <v>1</v>
       </c>
-      <c r="B57" s="22" t="e">
-        <f>DGET($A$1:$H$11,6.5,$G$25:$G$26)</f>
-        <v>#NUM!</v>
+      <c r="B57" s="22">
+        <f>DGET($A$1:$H$11,6.5,$A$14:$A$15)</f>
+        <v>11000</v>
       </c>
       <c r="C57" s="30" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="58" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A58" s="30">
         <v>1</v>
       </c>
-      <c r="B58" s="22" t="e">
-        <f>DGET($A$1:$H$11,6.0000001,$G$25:$G$26)</f>
-        <v>#NUM!</v>
+      <c r="B58" s="22">
+        <f>DGET($A$1:$H$11,6.0000001,$A$14:$A$15)</f>
+        <v>11000</v>
       </c>
       <c r="C58" s="30" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="59" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A59" s="5">
+      <c r="A59" s="30">
         <v>1</v>
       </c>
       <c r="B59" s="22" t="e">
-        <f>DGET($A$1:$H$11,6.9999999,$G$25:$G$26)</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="C59" s="30" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A60" s="30">
-        <v>1</v>
-      </c>
-      <c r="B60" s="22" t="e">
         <f>DGET($A$1:$H$11,$F$1,$A$14:$A$17)</f>
         <v>#NUM!</v>
       </c>
+      <c r="C59" s="30" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A60" s="5">
+        <v>28</v>
+      </c>
+      <c r="B60" s="22">
+        <f>DGET($A$1:$H$11,$F$1,$N$20:$N$21)</f>
+        <v>19800</v>
+      </c>
       <c r="C60" s="30" t="s">
         <v>129</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A61" s="5">
-        <v>28</v>
-      </c>
-      <c r="B61" s="22">
-        <f>DGET($A$1:$H$11,$F$1,$N$20:$N$21)</f>
-        <v>19800</v>
-      </c>
-      <c r="C61" s="30" t="s">
-        <v>130</v>
       </c>
     </row>
   </sheetData>
@@ -6864,7 +6837,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:Q69"/>
+  <dimension ref="A1:Q68"/>
   <sheetFormatPr defaultColWidth="12.59765625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="2" width="12.6640625" style="5" bestFit="1" customWidth="1"/>
@@ -6941,8 +6914,8 @@
       <c r="C2" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="34" t="s">
-        <v>123</v>
+      <c r="D2" s="35" t="s">
+        <v>15</v>
       </c>
       <c r="E2" s="34">
         <v>120</v>
@@ -6987,8 +6960,8 @@
       <c r="C3" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="34" t="s">
-        <v>124</v>
+      <c r="D3" s="35" t="s">
+        <v>21</v>
       </c>
       <c r="E3" s="34">
         <v>80</v>
@@ -7035,8 +7008,8 @@
       <c r="C4" s="34" t="s">
         <v>24</v>
       </c>
-      <c r="D4" s="34" t="s">
-        <v>123</v>
+      <c r="D4" s="35" t="s">
+        <v>15</v>
       </c>
       <c r="E4" s="34">
         <v>200</v>
@@ -7083,8 +7056,8 @@
       <c r="C5" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="34" t="s">
-        <v>123</v>
+      <c r="D5" s="35" t="s">
+        <v>15</v>
       </c>
       <c r="E5" s="34">
         <v>150</v>
@@ -7129,8 +7102,8 @@
       <c r="C6" s="34" t="s">
         <v>24</v>
       </c>
-      <c r="D6" s="34" t="s">
-        <v>124</v>
+      <c r="D6" s="35" t="s">
+        <v>21</v>
       </c>
       <c r="E6" s="34">
         <v>50</v>
@@ -7179,7 +7152,7 @@
       <c r="C7" s="34" t="s">
         <v>34</v>
       </c>
-      <c r="D7" s="34" t="s">
+      <c r="D7" s="35" t="s">
         <v>35</v>
       </c>
       <c r="E7" s="34">
@@ -7227,8 +7200,8 @@
       <c r="C8" s="34" t="s">
         <v>34</v>
       </c>
-      <c r="D8" s="34" t="s">
-        <v>123</v>
+      <c r="D8" s="35" t="s">
+        <v>15</v>
       </c>
       <c r="E8" s="34">
         <v>100</v>
@@ -7272,8 +7245,8 @@
       <c r="C9" s="34" t="s">
         <v>34</v>
       </c>
-      <c r="D9" s="34" t="s">
-        <v>123</v>
+      <c r="D9" s="35" t="s">
+        <v>15</v>
       </c>
       <c r="E9" s="34">
         <v>400</v>
@@ -7318,8 +7291,8 @@
       <c r="C10" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="D10" s="34" t="s">
-        <v>124</v>
+      <c r="D10" s="35" t="s">
+        <v>21</v>
       </c>
       <c r="E10" s="34">
         <v>250</v>
@@ -7369,8 +7342,8 @@
       <c r="C11" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="D11" s="34" t="s">
-        <v>123</v>
+      <c r="D11" s="35" t="s">
+        <v>15</v>
       </c>
       <c r="E11" s="34">
         <v>200</v>
@@ -7712,7 +7685,7 @@
     </row>
     <row r="23" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B23" s="21" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="J23" s="30"/>
       <c r="K23" s="30"/>
@@ -7826,7 +7799,7 @@
         <v>12</v>
       </c>
       <c r="N26" s="32" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="27" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.45">
@@ -7847,7 +7820,7 @@
       </c>
       <c r="B28" s="22">
         <f>DPRODUCT($A$1:$H$11,$F$1,E14:F15)</f>
-        <v>11000</v>
+        <v>0</v>
       </c>
       <c r="C28" s="5" t="s">
         <v>68</v>
@@ -7859,7 +7832,7 @@
       </c>
       <c r="B29" s="22">
         <f>DPRODUCT($A$1:$H$11,$F$1,G14:H16)</f>
-        <v>11000</v>
+        <v>0</v>
       </c>
       <c r="C29" s="5" t="s">
         <v>69</v>
@@ -7906,7 +7879,7 @@
         <v>10</v>
       </c>
       <c r="B33" s="29" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C33" s="28" t="s">
         <v>119</v>
@@ -8161,7 +8134,7 @@
         <v>0</v>
       </c>
       <c r="C54" s="30" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="55" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.45">
@@ -8266,7 +8239,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="C63" s="30" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="64" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.45">
@@ -8275,7 +8248,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="C64" s="30" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="65" spans="2:3" ht="15" customHeight="1" x14ac:dyDescent="0.45">
@@ -8284,7 +8257,7 @@
         <v>11000</v>
       </c>
       <c r="C65" s="30" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="66" spans="2:3" ht="15" customHeight="1" x14ac:dyDescent="0.45">
@@ -8293,34 +8266,25 @@
         <v>11000</v>
       </c>
       <c r="C66" s="30" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="67" spans="2:3" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B67" s="22">
-        <f>DPRODUCT($A$1:$P$11,6.9999999,$A$14:$A$15)</f>
-        <v>45503</v>
+        <f>DPRODUCT($A$1:$P$11,$F$1,$A$14:$A$17)</f>
+        <v>1.2356598988800001E+42</v>
       </c>
       <c r="C67" s="30" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
     </row>
     <row r="68" spans="2:3" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B68" s="22">
-        <f>DPRODUCT($A$1:$P$11,$F$1,$A$14:$A$17)</f>
-        <v>1.2356598988800001E+42</v>
+        <f>DPRODUCT($A$1:$P$11,$F$1,$N$25:$N$26)</f>
+        <v>475200000</v>
       </c>
       <c r="C68" s="30" t="s">
         <v>129</v>
-      </c>
-    </row>
-    <row r="69" spans="2:3" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B69" s="22">
-        <f>DPRODUCT($A$1:$P$11,$F$1,$N$25:$N$26)</f>
-        <v>475200000</v>
-      </c>
-      <c r="C69" s="30" t="s">
-        <v>130</v>
       </c>
     </row>
   </sheetData>

</xml_diff>